<commit_message>
fix: regras dos painéis conforme o Kayo
Positivação vira contagem distinta de cliente por fornecedor (atendimento
único do mês, qualquer vendedor); positivação do dia = primeira compra do
mês naquele dia. Todas as posições de pedido contam. Sábado é dia de venda.
Produtos foco: META é positivação e META II é financeiro, cada um com sua
barra e escala na TV.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015TKaSn4L8db77LPKSsZ5hm
</commit_message>
<xml_diff>
--- a/tools/exemplos/(BASE) - Metas Polybalas - Financeiro e Positivações.xlsx
+++ b/tools/exemplos/(BASE) - Metas Polybalas - Financeiro e Positivações.xlsx
@@ -487,7 +487,7 @@
         <v>3274.2793</v>
       </c>
       <c r="G2" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -516,7 +516,7 @@
         <v>8683.7268</v>
       </c>
       <c r="G3" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -542,10 +542,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>8246.778700000001</v>
+        <v>8090.0038</v>
       </c>
       <c r="G4" t="n">
-        <v>42</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -571,10 +571,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>7591.927</v>
+        <v>8246.778700000001</v>
       </c>
       <c r="G5" t="n">
-        <v>64</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
@@ -600,10 +600,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7381.6687</v>
+        <v>6406.6992</v>
       </c>
       <c r="G6" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>4059.5715</v>
+        <v>5233.9972</v>
       </c>
       <c r="G7" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8">
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>3219.7875</v>
+        <v>6060.7745</v>
       </c>
       <c r="G8" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -687,10 +687,10 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>5422.7564</v>
+        <v>7547.7218</v>
       </c>
       <c r="G9" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>6916.0281</v>
+        <v>7381.6687</v>
       </c>
       <c r="G10" t="n">
         <v>22</v>
@@ -745,10 +745,10 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>5081.9131</v>
+        <v>5367.1175</v>
       </c>
       <c r="G11" t="n">
-        <v>61</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12">
@@ -774,10 +774,10 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>8869.4303</v>
+        <v>6492.3278</v>
       </c>
       <c r="G12" t="n">
-        <v>61</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13">
@@ -803,10 +803,10 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>7733.3834</v>
+        <v>4367.0614</v>
       </c>
       <c r="G13" t="n">
-        <v>79</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -832,10 +832,10 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>6645.1635</v>
+        <v>5422.7564</v>
       </c>
       <c r="G14" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15">
@@ -861,10 +861,10 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>3082.8223</v>
+        <v>8291.2639</v>
       </c>
       <c r="G15" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16">
@@ -890,10 +890,10 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>4369.4126</v>
+        <v>6916.0281</v>
       </c>
       <c r="G16" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17">
@@ -919,10 +919,10 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>8197.086300000001</v>
+        <v>5081.9131</v>
       </c>
       <c r="G17" t="n">
-        <v>43</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18">
@@ -948,10 +948,10 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2660.8055</v>
+        <v>8869.4303</v>
       </c>
       <c r="G18" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19">
@@ -977,10 +977,10 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>4863.0245</v>
+        <v>4818.1343</v>
       </c>
       <c r="G19" t="n">
-        <v>55</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20">
@@ -1006,10 +1006,10 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>3089.4473</v>
+        <v>8997.764800000001</v>
       </c>
       <c r="G20" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21">
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>8136.9643</v>
+        <v>6645.1635</v>
       </c>
       <c r="G21" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22">
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5791.3319</v>
+        <v>4712.5647</v>
       </c>
       <c r="G22" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23">
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>5087.9647</v>
+        <v>5997.4207</v>
       </c>
       <c r="G23" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24">
@@ -1122,10 +1122,10 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>4181.1823</v>
+        <v>5473.4107</v>
       </c>
       <c r="G24" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25">
@@ -1151,10 +1151,10 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>6166.0008</v>
+        <v>6691.1678</v>
       </c>
       <c r="G25" t="n">
-        <v>46</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26">
@@ -1180,10 +1180,10 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>5834.1712</v>
+        <v>6253.2518</v>
       </c>
       <c r="G26" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27">
@@ -1209,10 +1209,10 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>6240.8556</v>
+        <v>8010.6628</v>
       </c>
       <c r="G27" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28">
@@ -1238,10 +1238,10 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>7817.8593</v>
+        <v>4863.0245</v>
       </c>
       <c r="G28" t="n">
-        <v>68</v>
+        <v>33</v>
       </c>
     </row>
     <row r="29">
@@ -1267,10 +1267,10 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>8264.3603</v>
+        <v>3089.4473</v>
       </c>
       <c r="G29" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30">
@@ -1296,10 +1296,10 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>7162.4989</v>
+        <v>6307.1658</v>
       </c>
       <c r="G30" t="n">
-        <v>35</v>
+        <v>21</v>
       </c>
     </row>
     <row r="31">
@@ -1325,10 +1325,10 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>5555.2621</v>
+        <v>8136.9643</v>
       </c>
       <c r="G31" t="n">
-        <v>38</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32">
@@ -1354,10 +1354,10 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>8247.99</v>
+        <v>5791.3319</v>
       </c>
       <c r="G32" t="n">
-        <v>34</v>
+        <v>50</v>
       </c>
     </row>
     <row r="33">
@@ -1383,10 +1383,10 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>6573.3583</v>
+        <v>8133.9058</v>
       </c>
       <c r="G33" t="n">
-        <v>74</v>
+        <v>54</v>
       </c>
     </row>
     <row r="34">
@@ -1412,10 +1412,10 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>6882.9706</v>
+        <v>5691.6996</v>
       </c>
       <c r="G34" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35">
@@ -1441,10 +1441,10 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>6138.6743</v>
+        <v>5910.2426</v>
       </c>
       <c r="G35" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="36">
@@ -1470,10 +1470,10 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>6062.9655</v>
+        <v>5229.78</v>
       </c>
       <c r="G36" t="n">
-        <v>53</v>
+        <v>36</v>
       </c>
     </row>
     <row r="37">
@@ -1499,10 +1499,10 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>7039.1031</v>
+        <v>8884.7124</v>
       </c>
       <c r="G37" t="n">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="38">
@@ -1528,10 +1528,10 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>5314.9344</v>
+        <v>5866.917</v>
       </c>
       <c r="G38" t="n">
-        <v>42</v>
+        <v>22</v>
       </c>
     </row>
     <row r="39">
@@ -1557,10 +1557,10 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>7906.973</v>
+        <v>6240.8556</v>
       </c>
       <c r="G39" t="n">
-        <v>17</v>
+        <v>39</v>
       </c>
     </row>
     <row r="40">
@@ -1586,10 +1586,10 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>2715.2102</v>
+        <v>3338.4925</v>
       </c>
       <c r="G40" t="n">
-        <v>57</v>
+        <v>22</v>
       </c>
     </row>
     <row r="41">
@@ -1615,10 +1615,10 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>7723.0551</v>
+        <v>8757.7142</v>
       </c>
       <c r="G41" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
     </row>
     <row r="42">
@@ -1644,10 +1644,10 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>4839.5831</v>
+        <v>8264.3603</v>
       </c>
       <c r="G42" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="43">
@@ -1673,10 +1673,10 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>4190.7184</v>
+        <v>7162.4989</v>
       </c>
       <c r="G43" t="n">
-        <v>34</v>
+        <v>18</v>
       </c>
     </row>
     <row r="44">
@@ -1702,10 +1702,10 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>5533.2647</v>
+        <v>5555.2621</v>
       </c>
       <c r="G44" t="n">
-        <v>47</v>
+        <v>25</v>
       </c>
     </row>
     <row r="45">
@@ -1731,10 +1731,10 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>7751.7353</v>
+        <v>8247.99</v>
       </c>
       <c r="G45" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="46">
@@ -1760,10 +1760,10 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>7904.119</v>
+        <v>8258.4879</v>
       </c>
       <c r="G46" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="47">
@@ -1789,10 +1789,10 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>5474.7613</v>
+        <v>7054.5976</v>
       </c>
       <c r="G47" t="n">
-        <v>27</v>
+        <v>39</v>
       </c>
     </row>
     <row r="48">
@@ -1818,10 +1818,10 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>5349.9318</v>
+        <v>5551.1392</v>
       </c>
       <c r="G48" t="n">
-        <v>66</v>
+        <v>45</v>
       </c>
     </row>
     <row r="49">
@@ -1847,10 +1847,10 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>4182.4025</v>
+        <v>8737.543299999999</v>
       </c>
       <c r="G49" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="50">
@@ -1876,10 +1876,10 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>8787.240599999999</v>
+        <v>4131.5421</v>
       </c>
       <c r="G50" t="n">
-        <v>38</v>
+        <v>20</v>
       </c>
     </row>
     <row r="51">
@@ -1905,10 +1905,10 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>8610.8956</v>
+        <v>6853.4006</v>
       </c>
       <c r="G51" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
     </row>
     <row r="52">
@@ -1934,10 +1934,10 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>8371.213900000001</v>
+        <v>6062.9655</v>
       </c>
       <c r="G52" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="53">
@@ -1963,10 +1963,10 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>3128.3065</v>
+        <v>5762.3475</v>
       </c>
       <c r="G53" t="n">
-        <v>68</v>
+        <v>41</v>
       </c>
     </row>
     <row r="54">
@@ -1992,10 +1992,10 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>3451.3314</v>
+        <v>7731.813</v>
       </c>
       <c r="G54" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
     </row>
     <row r="55">
@@ -2021,10 +2021,10 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>3099.0961</v>
+        <v>5314.9344</v>
       </c>
       <c r="G55" t="n">
-        <v>72</v>
+        <v>36</v>
       </c>
     </row>
     <row r="56">
@@ -2050,10 +2050,10 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>6274.1599</v>
+        <v>7906.973</v>
       </c>
       <c r="G56" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="57">
@@ -2079,10 +2079,10 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>6465.8692</v>
+        <v>2715.2102</v>
       </c>
       <c r="G57" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="58">
@@ -2108,10 +2108,10 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>4110.9445</v>
+        <v>8233.271000000001</v>
       </c>
       <c r="G58" t="n">
-        <v>17</v>
+        <v>28</v>
       </c>
     </row>
     <row r="59">
@@ -2137,10 +2137,10 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>7387.0575</v>
+        <v>7723.0551</v>
       </c>
       <c r="G59" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="60">
@@ -2166,10 +2166,10 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>6845.1014</v>
+        <v>5681.8639</v>
       </c>
       <c r="G60" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="61">
@@ -2195,10 +2195,10 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>3505.9459</v>
+        <v>3798.9442</v>
       </c>
       <c r="G61" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="62">
@@ -2224,10 +2224,10 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>6819.7786</v>
+        <v>5656.1994</v>
       </c>
       <c r="G62" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
     </row>
     <row r="63">
@@ -2253,10 +2253,10 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>6983.418</v>
+        <v>7483.5717</v>
       </c>
       <c r="G63" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="64">
@@ -2282,10 +2282,10 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>6047.7235</v>
+        <v>7751.7353</v>
       </c>
       <c r="G64" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
     </row>
     <row r="65">
@@ -2311,10 +2311,10 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>6321.5744</v>
+        <v>6815.334</v>
       </c>
       <c r="G65" t="n">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="66">
@@ -2340,10 +2340,10 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>4389.421</v>
+        <v>7904.119</v>
       </c>
       <c r="G66" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
     </row>
     <row r="67">
@@ -2369,10 +2369,10 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>6845.6067</v>
+        <v>5474.7613</v>
       </c>
       <c r="G67" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
     </row>
     <row r="68">
@@ -2398,10 +2398,10 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>7592.3467</v>
+        <v>3139.4309</v>
       </c>
       <c r="G68" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="69">
@@ -2427,10 +2427,10 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>5800.0623</v>
+        <v>7157.3699</v>
       </c>
       <c r="G69" t="n">
-        <v>54</v>
+        <v>36</v>
       </c>
     </row>
     <row r="70">
@@ -2456,10 +2456,10 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>7751.9675</v>
+        <v>4182.4025</v>
       </c>
       <c r="G70" t="n">
-        <v>68</v>
+        <v>45</v>
       </c>
     </row>
     <row r="71">
@@ -2485,10 +2485,10 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>7744.9005</v>
+        <v>8774.2433</v>
       </c>
       <c r="G71" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
     </row>
     <row r="72">
@@ -2514,10 +2514,10 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>2591.8572</v>
+        <v>7975.8585</v>
       </c>
       <c r="G72" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="73">
@@ -2543,10 +2543,10 @@
         </is>
       </c>
       <c r="F73" t="n">
-        <v>5030.7619</v>
+        <v>8610.8956</v>
       </c>
       <c r="G73" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
     </row>
     <row r="74">
@@ -2572,10 +2572,10 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>2833.9399</v>
+        <v>4232.0299</v>
       </c>
       <c r="G74" t="n">
-        <v>61</v>
+        <v>41</v>
       </c>
     </row>
     <row r="75">
@@ -2601,10 +2601,10 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>6700.7709</v>
+        <v>4905.837</v>
       </c>
       <c r="G75" t="n">
-        <v>23</v>
+        <v>34</v>
       </c>
     </row>
     <row r="76">
@@ -2630,10 +2630,10 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>2666.2849</v>
+        <v>7359.0836</v>
       </c>
       <c r="G76" t="n">
-        <v>76</v>
+        <v>40</v>
       </c>
     </row>
     <row r="77">
@@ -2659,10 +2659,10 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>4630.4403</v>
+        <v>3451.3314</v>
       </c>
       <c r="G77" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="78">
@@ -2688,10 +2688,10 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>5425.9125</v>
+        <v>2591.2115</v>
       </c>
       <c r="G78" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="79">
@@ -2717,10 +2717,10 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>5734.2029</v>
+        <v>5432.9971</v>
       </c>
       <c r="G79" t="n">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="80">
@@ -2746,10 +2746,10 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>6215.5184</v>
+        <v>8559.1592</v>
       </c>
       <c r="G80" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
     </row>
     <row r="81">
@@ -2775,10 +2775,10 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>3500.2888</v>
+        <v>6465.8692</v>
       </c>
       <c r="G81" t="n">
-        <v>63</v>
+        <v>27</v>
       </c>
     </row>
     <row r="82">
@@ -2804,10 +2804,10 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>3845.4067</v>
+        <v>4110.9445</v>
       </c>
       <c r="G82" t="n">
-        <v>46</v>
+        <v>35</v>
       </c>
     </row>
     <row r="83">
@@ -2833,10 +2833,10 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>5482.3122</v>
+        <v>2790.284</v>
       </c>
       <c r="G83" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="84">
@@ -2862,10 +2862,10 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>6910.239</v>
+        <v>8716.3848</v>
       </c>
       <c r="G84" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
     </row>
     <row r="85">
@@ -2891,10 +2891,10 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>6057.8007</v>
+        <v>7424.7992</v>
       </c>
       <c r="G85" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="86">
@@ -2920,10 +2920,10 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>3770.7106</v>
+        <v>3505.9459</v>
       </c>
       <c r="G86" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="87">
@@ -2949,10 +2949,10 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>2794.0379</v>
+        <v>6819.7786</v>
       </c>
       <c r="G87" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
     </row>
     <row r="88">
@@ -2978,10 +2978,10 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>5436.8356</v>
+        <v>7501.9308</v>
       </c>
       <c r="G88" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="89">
@@ -3007,10 +3007,10 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>5644.9651</v>
+        <v>5697.928</v>
       </c>
       <c r="G89" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="90">
@@ -3036,10 +3036,10 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>3339.4086</v>
+        <v>8593.838100000001</v>
       </c>
       <c r="G90" t="n">
-        <v>68</v>
+        <v>36</v>
       </c>
     </row>
     <row r="91">
@@ -3065,10 +3065,10 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>3921.703</v>
+        <v>3949.0299</v>
       </c>
       <c r="G91" t="n">
-        <v>68</v>
+        <v>38</v>
       </c>
     </row>
     <row r="92">
@@ -3094,10 +3094,10 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>8315.002</v>
+        <v>3352.9058</v>
       </c>
       <c r="G92" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="93">
@@ -3123,10 +3123,10 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>3542.5394</v>
+        <v>8193.959699999999</v>
       </c>
       <c r="G93" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="94">
@@ -3152,10 +3152,10 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>5034.8143</v>
+        <v>4389.421</v>
       </c>
       <c r="G94" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
     </row>
     <row r="95">
@@ -3181,10 +3181,10 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>5964.5709</v>
+        <v>6845.6067</v>
       </c>
       <c r="G95" t="n">
-        <v>31</v>
+        <v>54</v>
       </c>
     </row>
     <row r="96">
@@ -3210,10 +3210,10 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>4990.7047</v>
+        <v>3379.7499</v>
       </c>
       <c r="G96" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
     </row>
     <row r="97">
@@ -3239,10 +3239,10 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>4736.4288</v>
+        <v>8447.6049</v>
       </c>
       <c r="G97" t="n">
-        <v>50</v>
+        <v>36</v>
       </c>
     </row>
     <row r="98">
@@ -3268,10 +3268,10 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>5515.4492</v>
+        <v>5800.0623</v>
       </c>
       <c r="G98" t="n">
-        <v>46</v>
+        <v>26</v>
       </c>
     </row>
     <row r="99">
@@ -3297,10 +3297,10 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>4369.8567</v>
+        <v>7751.9675</v>
       </c>
       <c r="G99" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="100">
@@ -3326,10 +3326,10 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>4617.6302</v>
+        <v>7744.9005</v>
       </c>
       <c r="G100" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
     </row>
     <row r="101">
@@ -3355,10 +3355,10 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>5389.7888</v>
+        <v>2591.8572</v>
       </c>
       <c r="G101" t="n">
-        <v>63</v>
+        <v>24</v>
       </c>
     </row>
     <row r="102">
@@ -3384,10 +3384,10 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>7677.916</v>
+        <v>5030.7619</v>
       </c>
       <c r="G102" t="n">
-        <v>41</v>
+        <v>24</v>
       </c>
     </row>
     <row r="103">
@@ -3413,10 +3413,10 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>7804.9902</v>
+        <v>2833.9399</v>
       </c>
       <c r="G103" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="104">
@@ -3442,10 +3442,10 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>4003.6763</v>
+        <v>6700.7709</v>
       </c>
       <c r="G104" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="105">
@@ -3471,10 +3471,10 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>8211.035</v>
+        <v>7501.9693</v>
       </c>
       <c r="G105" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="106">
@@ -3500,7 +3500,7 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>5152.016</v>
+        <v>2666.2849</v>
       </c>
       <c r="G106" t="n">
         <v>18</v>
@@ -3529,10 +3529,10 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>8747.790999999999</v>
+        <v>4630.4403</v>
       </c>
       <c r="G107" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
     </row>
     <row r="108">
@@ -3558,10 +3558,10 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>8002.5119</v>
+        <v>5425.9125</v>
       </c>
       <c r="G108" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="109">
@@ -3587,10 +3587,10 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>6153.0165</v>
+        <v>3288.9235</v>
       </c>
       <c r="G109" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="110">
@@ -3616,10 +3616,10 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>3213.0078</v>
+        <v>6215.5184</v>
       </c>
       <c r="G110" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="111">
@@ -3645,7 +3645,7 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>6112.6984</v>
+        <v>3609.7684</v>
       </c>
       <c r="G111" t="n">
         <v>38</v>
@@ -3674,10 +3674,10 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>6203.9276</v>
+        <v>5877.4892</v>
       </c>
       <c r="G112" t="n">
-        <v>44</v>
+        <v>33</v>
       </c>
     </row>
     <row r="113">
@@ -3703,10 +3703,10 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>6856.9979</v>
+        <v>6551.7299</v>
       </c>
       <c r="G113" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="114">
@@ -3732,10 +3732,10 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>3159.4623</v>
+        <v>6388.4274</v>
       </c>
       <c r="G114" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="115">
@@ -3761,10 +3761,10 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>3126.7998</v>
+        <v>7120.7374</v>
       </c>
       <c r="G115" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
     </row>
     <row r="116">
@@ -3790,10 +3790,10 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>3613.2881</v>
+        <v>5094.521</v>
       </c>
       <c r="G116" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
     </row>
     <row r="117">
@@ -3819,10 +3819,10 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>7434.2328</v>
+        <v>6706.998</v>
       </c>
       <c r="G117" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="118">
@@ -3848,10 +3848,10 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>6698.6385</v>
+        <v>2794.0379</v>
       </c>
       <c r="G118" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
     </row>
     <row r="119">
@@ -3877,10 +3877,10 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>5793.0735</v>
+        <v>8551.2191</v>
       </c>
       <c r="G119" t="n">
-        <v>35</v>
+        <v>19</v>
       </c>
     </row>
     <row r="120">
@@ -3906,10 +3906,10 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>6322.7056</v>
+        <v>5436.8356</v>
       </c>
       <c r="G120" t="n">
-        <v>19</v>
+        <v>34</v>
       </c>
     </row>
     <row r="121">
@@ -3935,10 +3935,10 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>4391.735</v>
+        <v>6665.5427</v>
       </c>
       <c r="G121" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="122">
@@ -3964,10 +3964,10 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>3549.0407</v>
+        <v>7121.1457</v>
       </c>
       <c r="G122" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="123">
@@ -3993,10 +3993,10 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>2908.714</v>
+        <v>2633.0539</v>
       </c>
       <c r="G123" t="n">
-        <v>53</v>
+        <v>36</v>
       </c>
     </row>
     <row r="124">
@@ -4022,7 +4022,7 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>8132.2079</v>
+        <v>5944.5876</v>
       </c>
       <c r="G124" t="n">
         <v>39</v>
@@ -4051,10 +4051,10 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>5194.4337</v>
+        <v>8237.3313</v>
       </c>
       <c r="G125" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
     </row>
     <row r="126">
@@ -4080,10 +4080,10 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>2872.5255</v>
+        <v>8717.818499999999</v>
       </c>
       <c r="G126" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="127">
@@ -4109,10 +4109,10 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>2649.3551</v>
+        <v>6797.949</v>
       </c>
       <c r="G127" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="128">
@@ -4138,10 +4138,10 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>3110.1559</v>
+        <v>5034.8143</v>
       </c>
       <c r="G128" t="n">
-        <v>37</v>
+        <v>24</v>
       </c>
     </row>
     <row r="129">
@@ -4167,10 +4167,10 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>4547.3338</v>
+        <v>5964.5709</v>
       </c>
       <c r="G129" t="n">
-        <v>45</v>
+        <v>32</v>
       </c>
     </row>
     <row r="130">
@@ -4196,10 +4196,10 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>6447.1579</v>
+        <v>3011.2823</v>
       </c>
       <c r="G130" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="131">
@@ -4225,10 +4225,10 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>8510.8357</v>
+        <v>3716.7921</v>
       </c>
       <c r="G131" t="n">
-        <v>48</v>
+        <v>27</v>
       </c>
     </row>
     <row r="132">
@@ -4254,10 +4254,10 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>6450.6067</v>
+        <v>4212.384</v>
       </c>
       <c r="G132" t="n">
-        <v>62</v>
+        <v>34</v>
       </c>
     </row>
     <row r="133">
@@ -4283,10 +4283,10 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>5269.8058</v>
+        <v>8995.0818</v>
       </c>
       <c r="G133" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
     </row>
     <row r="134">
@@ -4312,10 +4312,10 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>6962.0125</v>
+        <v>5202.2931</v>
       </c>
       <c r="G134" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
     </row>
     <row r="135">
@@ -4341,10 +4341,10 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>6929.124</v>
+        <v>3650.2548</v>
       </c>
       <c r="G135" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="136">
@@ -4370,10 +4370,10 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>5028.8075</v>
+        <v>5633.3431</v>
       </c>
       <c r="G136" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
     </row>
     <row r="137">
@@ -4399,10 +4399,10 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>2874.5997</v>
+        <v>5927.137</v>
       </c>
       <c r="G137" t="n">
-        <v>70</v>
+        <v>43</v>
       </c>
     </row>
     <row r="138">
@@ -4428,10 +4428,10 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>8209.713299999999</v>
+        <v>7678.628</v>
       </c>
       <c r="G138" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="139">
@@ -4457,10 +4457,10 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>7019.4541</v>
+        <v>3114.6793</v>
       </c>
       <c r="G139" t="n">
-        <v>54</v>
+        <v>34</v>
       </c>
     </row>
     <row r="140">
@@ -4486,10 +4486,10 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>7226.3232</v>
+        <v>4003.6763</v>
       </c>
       <c r="G140" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="141">
@@ -4515,10 +4515,10 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>4430.1232</v>
+        <v>8211.035</v>
       </c>
       <c r="G141" t="n">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="142">
@@ -4544,10 +4544,10 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>4572.7364</v>
+        <v>4647.874</v>
       </c>
       <c r="G142" t="n">
-        <v>16</v>
+        <v>29</v>
       </c>
     </row>
     <row r="143">
@@ -4573,10 +4573,10 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>6024.0194</v>
+        <v>7591.54</v>
       </c>
       <c r="G143" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="144">
@@ -4602,10 +4602,10 @@
         </is>
       </c>
       <c r="F144" t="n">
-        <v>3783.4139</v>
+        <v>8001.69</v>
       </c>
       <c r="G144" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="145">
@@ -4631,10 +4631,10 @@
         </is>
       </c>
       <c r="F145" t="n">
-        <v>7190.9085</v>
+        <v>8747.790999999999</v>
       </c>
       <c r="G145" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="146">
@@ -4660,10 +4660,10 @@
         </is>
       </c>
       <c r="F146" t="n">
-        <v>3553.8069</v>
+        <v>8002.5119</v>
       </c>
       <c r="G146" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="147">
@@ -4689,10 +4689,10 @@
         </is>
       </c>
       <c r="F147" t="n">
-        <v>3268.8392</v>
+        <v>6153.0165</v>
       </c>
       <c r="G147" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="148">
@@ -4718,10 +4718,10 @@
         </is>
       </c>
       <c r="F148" t="n">
-        <v>5896.7953</v>
+        <v>7646.7195</v>
       </c>
       <c r="G148" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="149">
@@ -4747,10 +4747,10 @@
         </is>
       </c>
       <c r="F149" t="n">
-        <v>2687.1621</v>
+        <v>3213.0078</v>
       </c>
       <c r="G149" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
     </row>
     <row r="150">
@@ -4776,10 +4776,10 @@
         </is>
       </c>
       <c r="F150" t="n">
-        <v>4813.8144</v>
+        <v>4323.0698</v>
       </c>
       <c r="G150" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
     </row>
     <row r="151">
@@ -4805,10 +4805,10 @@
         </is>
       </c>
       <c r="F151" t="n">
-        <v>4951.6841</v>
+        <v>6192.2699</v>
       </c>
       <c r="G151" t="n">
-        <v>42</v>
+        <v>21</v>
       </c>
     </row>
     <row r="152">
@@ -4834,10 +4834,10 @@
         </is>
       </c>
       <c r="F152" t="n">
-        <v>6806.8547</v>
+        <v>6203.9276</v>
       </c>
       <c r="G152" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
     </row>
     <row r="153">
@@ -4863,10 +4863,10 @@
         </is>
       </c>
       <c r="F153" t="n">
-        <v>3692.5363</v>
+        <v>4242.6546</v>
       </c>
       <c r="G153" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
     </row>
     <row r="154">
@@ -4892,10 +4892,10 @@
         </is>
       </c>
       <c r="F154" t="n">
-        <v>6800.1575</v>
+        <v>3362.018</v>
       </c>
       <c r="G154" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
     </row>
     <row r="155">
@@ -4921,10 +4921,10 @@
         </is>
       </c>
       <c r="F155" t="n">
-        <v>8279.449500000001</v>
+        <v>4214.1327</v>
       </c>
       <c r="G155" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="156">
@@ -4950,10 +4950,10 @@
         </is>
       </c>
       <c r="F156" t="n">
-        <v>3983.6627</v>
+        <v>3613.2881</v>
       </c>
       <c r="G156" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
     </row>
     <row r="157">
@@ -4979,10 +4979,10 @@
         </is>
       </c>
       <c r="F157" t="n">
-        <v>4299.4052</v>
+        <v>2892.7697</v>
       </c>
       <c r="G157" t="n">
-        <v>38</v>
+        <v>19</v>
       </c>
     </row>
     <row r="158">
@@ -5008,10 +5008,10 @@
         </is>
       </c>
       <c r="F158" t="n">
-        <v>5216.2185</v>
+        <v>7195.329</v>
       </c>
       <c r="G158" t="n">
-        <v>58</v>
+        <v>32</v>
       </c>
     </row>
     <row r="159">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="F159" t="n">
-        <v>3401.2734</v>
+        <v>6698.6385</v>
       </c>
       <c r="G159" t="n">
         <v>31</v>
@@ -5066,10 +5066,10 @@
         </is>
       </c>
       <c r="F160" t="n">
-        <v>7957.0964</v>
+        <v>5793.0735</v>
       </c>
       <c r="G160" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
     </row>
     <row r="161">
@@ -5095,10 +5095,10 @@
         </is>
       </c>
       <c r="F161" t="n">
-        <v>6726.386</v>
+        <v>6322.7056</v>
       </c>
       <c r="G161" t="n">
-        <v>53</v>
+        <v>20</v>
       </c>
     </row>
     <row r="162">
@@ -5124,10 +5124,10 @@
         </is>
       </c>
       <c r="F162" t="n">
-        <v>7829.1116</v>
+        <v>4391.735</v>
       </c>
       <c r="G162" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="163">
@@ -5153,10 +5153,10 @@
         </is>
       </c>
       <c r="F163" t="n">
-        <v>6614.5426</v>
+        <v>3549.0407</v>
       </c>
       <c r="G163" t="n">
-        <v>38</v>
+        <v>24</v>
       </c>
     </row>
     <row r="164">
@@ -5182,10 +5182,10 @@
         </is>
       </c>
       <c r="F164" t="n">
-        <v>2865.6623</v>
+        <v>2908.714</v>
       </c>
       <c r="G164" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
     </row>
     <row r="165">
@@ -5211,10 +5211,10 @@
         </is>
       </c>
       <c r="F165" t="n">
-        <v>6581.078</v>
+        <v>8132.2079</v>
       </c>
       <c r="G165" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="166">
@@ -5240,10 +5240,10 @@
         </is>
       </c>
       <c r="F166" t="n">
-        <v>5558.5429</v>
+        <v>7549.0654</v>
       </c>
       <c r="G166" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="167">
@@ -5269,10 +5269,10 @@
         </is>
       </c>
       <c r="F167" t="n">
-        <v>6914.4308</v>
+        <v>8775.312900000001</v>
       </c>
       <c r="G167" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="168">
@@ -5298,10 +5298,10 @@
         </is>
       </c>
       <c r="F168" t="n">
-        <v>8526.9925</v>
+        <v>3126.9244</v>
       </c>
       <c r="G168" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
     </row>
     <row r="169">
@@ -5327,10 +5327,10 @@
         </is>
       </c>
       <c r="F169" t="n">
-        <v>7097.2523</v>
+        <v>4514.4714</v>
       </c>
       <c r="G169" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
     </row>
     <row r="170">
@@ -5356,10 +5356,10 @@
         </is>
       </c>
       <c r="F170" t="n">
-        <v>8681.499400000001</v>
+        <v>6957.8723</v>
       </c>
       <c r="G170" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="171">
@@ -5385,7 +5385,7 @@
         </is>
       </c>
       <c r="F171" t="n">
-        <v>6150.3365</v>
+        <v>8922.5173</v>
       </c>
       <c r="G171" t="n">
         <v>32</v>
@@ -5414,10 +5414,10 @@
         </is>
       </c>
       <c r="F172" t="n">
-        <v>4733.9717</v>
+        <v>4776.9943</v>
       </c>
       <c r="G172" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="173">
@@ -5443,10 +5443,10 @@
         </is>
       </c>
       <c r="F173" t="n">
-        <v>4935.7224</v>
+        <v>5464.2906</v>
       </c>
       <c r="G173" t="n">
-        <v>62</v>
+        <v>39</v>
       </c>
     </row>
     <row r="174">
@@ -5472,10 +5472,10 @@
         </is>
       </c>
       <c r="F174" t="n">
-        <v>6640.5741</v>
+        <v>6755.6612</v>
       </c>
       <c r="G174" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
     </row>
     <row r="175">
@@ -5501,10 +5501,10 @@
         </is>
       </c>
       <c r="F175" t="n">
-        <v>8330.6448</v>
+        <v>2747.0706</v>
       </c>
       <c r="G175" t="n">
-        <v>46</v>
+        <v>33</v>
       </c>
     </row>
     <row r="176">
@@ -5530,10 +5530,10 @@
         </is>
       </c>
       <c r="F176" t="n">
-        <v>3721.3648</v>
+        <v>4554.4142</v>
       </c>
       <c r="G176" t="n">
-        <v>34</v>
+        <v>17</v>
       </c>
     </row>
     <row r="177">
@@ -5559,10 +5559,10 @@
         </is>
       </c>
       <c r="F177" t="n">
-        <v>3499.5676</v>
+        <v>6361.3734</v>
       </c>
       <c r="G177" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
     </row>
     <row r="178">
@@ -5588,10 +5588,10 @@
         </is>
       </c>
       <c r="F178" t="n">
-        <v>8677.875700000001</v>
+        <v>8864.228800000001</v>
       </c>
       <c r="G178" t="n">
-        <v>40</v>
+        <v>27</v>
       </c>
     </row>
     <row r="179">
@@ -5617,10 +5617,10 @@
         </is>
       </c>
       <c r="F179" t="n">
-        <v>7065.2659</v>
+        <v>3276.3617</v>
       </c>
       <c r="G179" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
     </row>
     <row r="180">
@@ -5646,10 +5646,10 @@
         </is>
       </c>
       <c r="F180" t="n">
-        <v>6654.2561</v>
+        <v>8098.455</v>
       </c>
       <c r="G180" t="n">
-        <v>31</v>
+        <v>47</v>
       </c>
     </row>
     <row r="181">
@@ -5675,10 +5675,10 @@
         </is>
       </c>
       <c r="F181" t="n">
-        <v>4443.7353</v>
+        <v>8832.8768</v>
       </c>
       <c r="G181" t="n">
-        <v>50</v>
+        <v>36</v>
       </c>
     </row>
     <row r="182">
@@ -5704,10 +5704,10 @@
         </is>
       </c>
       <c r="F182" t="n">
-        <v>3396.7438</v>
+        <v>5028.8075</v>
       </c>
       <c r="G182" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
     </row>
     <row r="183">
@@ -5733,10 +5733,10 @@
         </is>
       </c>
       <c r="F183" t="n">
-        <v>8992.273499999999</v>
+        <v>4816.0664</v>
       </c>
       <c r="G183" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
     </row>
     <row r="184">
@@ -5762,10 +5762,10 @@
         </is>
       </c>
       <c r="F184" t="n">
-        <v>5967.2011</v>
+        <v>7148.6224</v>
       </c>
       <c r="G184" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="185">
@@ -5791,10 +5791,10 @@
         </is>
       </c>
       <c r="F185" t="n">
-        <v>6222.0907</v>
+        <v>2653.8115</v>
       </c>
       <c r="G185" t="n">
-        <v>52</v>
+        <v>38</v>
       </c>
     </row>
     <row r="186">
@@ -5820,10 +5820,10 @@
         </is>
       </c>
       <c r="F186" t="n">
-        <v>4973.7821</v>
+        <v>4648.5623</v>
       </c>
       <c r="G186" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
     </row>
     <row r="187">
@@ -5849,10 +5849,10 @@
         </is>
       </c>
       <c r="F187" t="n">
-        <v>7778.3036</v>
+        <v>8728.8475</v>
       </c>
       <c r="G187" t="n">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="188">
@@ -5878,10 +5878,10 @@
         </is>
       </c>
       <c r="F188" t="n">
-        <v>8773.544099999999</v>
+        <v>8453.0982</v>
       </c>
       <c r="G188" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="189">
@@ -5907,10 +5907,10 @@
         </is>
       </c>
       <c r="F189" t="n">
-        <v>3055.9887</v>
+        <v>7491.3072</v>
       </c>
       <c r="G189" t="n">
-        <v>29</v>
+        <v>17</v>
       </c>
     </row>
     <row r="190">
@@ -5936,10 +5936,10 @@
         </is>
       </c>
       <c r="F190" t="n">
-        <v>4668.4646</v>
+        <v>6306.4395</v>
       </c>
       <c r="G190" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="191">
@@ -5965,10 +5965,10 @@
         </is>
       </c>
       <c r="F191" t="n">
-        <v>4517.7285</v>
+        <v>6024.0194</v>
       </c>
       <c r="G191" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="192">
@@ -5994,10 +5994,10 @@
         </is>
       </c>
       <c r="F192" t="n">
-        <v>3554.3693</v>
+        <v>3783.4139</v>
       </c>
       <c r="G192" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
     </row>
     <row r="193">
@@ -6023,10 +6023,10 @@
         </is>
       </c>
       <c r="F193" t="n">
-        <v>4419.397</v>
+        <v>7190.9085</v>
       </c>
       <c r="G193" t="n">
-        <v>33</v>
+        <v>19</v>
       </c>
     </row>
     <row r="194">
@@ -6052,10 +6052,10 @@
         </is>
       </c>
       <c r="F194" t="n">
-        <v>4821.9516</v>
+        <v>3553.8069</v>
       </c>
       <c r="G194" t="n">
-        <v>54</v>
+        <v>26</v>
       </c>
     </row>
     <row r="195">
@@ -6081,10 +6081,10 @@
         </is>
       </c>
       <c r="F195" t="n">
-        <v>3726.5315</v>
+        <v>3268.8392</v>
       </c>
       <c r="G195" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="196">
@@ -6110,10 +6110,10 @@
         </is>
       </c>
       <c r="F196" t="n">
-        <v>8007.5088</v>
+        <v>5896.7953</v>
       </c>
       <c r="G196" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
     </row>
     <row r="197">
@@ -6139,10 +6139,10 @@
         </is>
       </c>
       <c r="F197" t="n">
-        <v>8604.9125</v>
+        <v>6711.3075</v>
       </c>
       <c r="G197" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="198">
@@ -6168,7 +6168,7 @@
         </is>
       </c>
       <c r="F198" t="n">
-        <v>7778.8341</v>
+        <v>4464.5676</v>
       </c>
       <c r="G198" t="n">
         <v>20</v>
@@ -6197,10 +6197,10 @@
         </is>
       </c>
       <c r="F199" t="n">
-        <v>7192.8712</v>
+        <v>6257.8265</v>
       </c>
       <c r="G199" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="200">
@@ -6226,10 +6226,10 @@
         </is>
       </c>
       <c r="F200" t="n">
-        <v>3667.5502</v>
+        <v>5199.4376</v>
       </c>
       <c r="G200" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="201">
@@ -6255,10 +6255,10 @@
         </is>
       </c>
       <c r="F201" t="n">
-        <v>3565.597</v>
+        <v>4055.4889</v>
       </c>
       <c r="G201" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="202">
@@ -6284,10 +6284,10 @@
         </is>
       </c>
       <c r="F202" t="n">
-        <v>5847.4493</v>
+        <v>6806.8547</v>
       </c>
       <c r="G202" t="n">
-        <v>22</v>
+        <v>50</v>
       </c>
     </row>
     <row r="203">
@@ -6313,10 +6313,10 @@
         </is>
       </c>
       <c r="F203" t="n">
-        <v>7972.4348</v>
+        <v>3313.8524</v>
       </c>
       <c r="G203" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="204">
@@ -6342,10 +6342,10 @@
         </is>
       </c>
       <c r="F204" t="n">
-        <v>4891.9775</v>
+        <v>2684.7113</v>
       </c>
       <c r="G204" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="205">
@@ -6371,10 +6371,10 @@
         </is>
       </c>
       <c r="F205" t="n">
-        <v>5958.8585</v>
+        <v>8575.325500000001</v>
       </c>
       <c r="G205" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="206">
@@ -6400,10 +6400,10 @@
         </is>
       </c>
       <c r="F206" t="n">
-        <v>3322.409</v>
+        <v>6106.8379</v>
       </c>
       <c r="G206" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="207">
@@ -6429,10 +6429,10 @@
         </is>
       </c>
       <c r="F207" t="n">
-        <v>5649.6712</v>
+        <v>4157.333</v>
       </c>
       <c r="G207" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="208">
@@ -6458,10 +6458,10 @@
         </is>
       </c>
       <c r="F208" t="n">
-        <v>4977.7907</v>
+        <v>3983.6627</v>
       </c>
       <c r="G208" t="n">
-        <v>43</v>
+        <v>22</v>
       </c>
     </row>
     <row r="209">
@@ -6487,10 +6487,10 @@
         </is>
       </c>
       <c r="F209" t="n">
-        <v>6709.0463</v>
+        <v>4299.4052</v>
       </c>
       <c r="G209" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="210">
@@ -6516,10 +6516,10 @@
         </is>
       </c>
       <c r="F210" t="n">
-        <v>5583.4764</v>
+        <v>5216.2185</v>
       </c>
       <c r="G210" t="n">
-        <v>34</v>
+        <v>17</v>
       </c>
     </row>
     <row r="211">
@@ -6545,10 +6545,10 @@
         </is>
       </c>
       <c r="F211" t="n">
-        <v>3286.1011</v>
+        <v>3401.2734</v>
       </c>
       <c r="G211" t="n">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>